<commit_message>
Replace repository with current project files
</commit_message>
<xml_diff>
--- a/result/batch123/F3F4.xlsx
+++ b/result/batch123/F3F4.xlsx
@@ -4,11 +4,11 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="17655" activeTab="3"/>
+    <workbookView windowHeight="17655" activeTab="4"/>
   </bookViews>
   <sheets>
-    <sheet name="F3a" sheetId="2" r:id="rId1"/>
-    <sheet name="F3b" sheetId="1" r:id="rId2"/>
+    <sheet name="F3a" sheetId="1" r:id="rId1"/>
+    <sheet name="F3b" sheetId="2" r:id="rId2"/>
     <sheet name="F4a" sheetId="3" r:id="rId3"/>
     <sheet name="F4b" sheetId="4" r:id="rId4"/>
     <sheet name="F4c" sheetId="5" r:id="rId5"/>
@@ -31,18 +31,30 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="8">
+  <si>
+    <t>0.0001</t>
+  </si>
+  <si>
+    <t>0.001</t>
+  </si>
+  <si>
+    <t>0.002</t>
+  </si>
+  <si>
+    <t>0.01</t>
+  </si>
+  <si>
+    <t>0.1</t>
+  </si>
+  <si>
+    <t>0.2</t>
+  </si>
   <si>
     <t>C</t>
   </si>
   <si>
     <t>M</t>
-  </si>
-  <si>
-    <t>C1</t>
-  </si>
-  <si>
-    <t>M1</t>
   </si>
 </sst>
 </file>
@@ -64,8 +76,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <b/>
+      <sz val="11"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -421,12 +433,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -532,158 +559,164 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="34" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1213,28 +1246,28 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="2" outlineLevelCol="6"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="B1">
-        <v>0.0001</v>
-      </c>
-      <c r="C1">
-        <v>0.001</v>
-      </c>
-      <c r="D1">
-        <v>0.002</v>
-      </c>
-      <c r="E1">
-        <v>0.01</v>
-      </c>
-      <c r="F1">
-        <v>0.1</v>
-      </c>
-      <c r="G1">
-        <v>0.2</v>
+      <c r="B1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" t="s">
-        <v>0</v>
+      <c r="A2" s="5" t="s">
+        <v>6</v>
       </c>
       <c r="B2">
         <v>0.13</v>
@@ -1256,8 +1289,8 @@
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" t="s">
-        <v>1</v>
+      <c r="A3" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B3">
         <v>0.81</v>
@@ -1288,31 +1321,31 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultColWidth="8.725" defaultRowHeight="13.5" outlineLevelRow="2" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="2" outlineLevelCol="6"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="B1">
-        <v>0.0001</v>
-      </c>
-      <c r="C1">
-        <v>0.001</v>
-      </c>
-      <c r="D1">
-        <v>0.002</v>
-      </c>
-      <c r="E1">
-        <v>0.01</v>
-      </c>
-      <c r="F1">
-        <v>0.1</v>
-      </c>
-      <c r="G1">
-        <v>0.2</v>
+      <c r="B1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" t="s">
-        <v>0</v>
+      <c r="A2" s="5" t="s">
+        <v>6</v>
       </c>
       <c r="B2">
         <v>0.224</v>
@@ -1321,7 +1354,7 @@
         <v>-0.035</v>
       </c>
       <c r="D2">
-        <v>0.609</v>
+        <v>0.565</v>
       </c>
       <c r="E2">
         <v>0.441</v>
@@ -1334,14 +1367,14 @@
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" t="s">
-        <v>1</v>
+      <c r="A3" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="B3">
         <v>1.995</v>
       </c>
       <c r="C3">
-        <v>2.312</v>
+        <v>2.321</v>
       </c>
       <c r="D3">
         <v>2.941</v>
@@ -1365,119 +1398,74 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="5" outlineLevelCol="6"/>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="2" outlineLevelCol="6"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="B1">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1">
         <v>0.0001</v>
       </c>
-      <c r="C1">
+      <c r="C1" s="1">
         <v>0.001</v>
       </c>
-      <c r="D1">
+      <c r="D1" s="1">
         <v>0.002</v>
       </c>
-      <c r="E1">
+      <c r="E1" s="1">
         <v>0.01</v>
       </c>
-      <c r="F1">
+      <c r="F1" s="1">
         <v>0.1</v>
       </c>
-      <c r="G1">
+      <c r="G1" s="1">
         <v>0.2</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="2">
         <v>0.093</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="2">
         <v>0.074</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="2">
         <v>0.092</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="4">
         <v>0.256</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F2" s="3">
         <v>0.485</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2" s="2">
         <v>0.144</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="1">
+      <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="2">
         <v>0.828</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="3">
         <v>1.689</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="2">
         <v>1.047</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>1.259</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3" s="2">
         <v>0.135</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3" s="2">
         <v>0.318</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5">
-        <v>0.074</v>
-      </c>
-      <c r="C5">
-        <v>0.256</v>
-      </c>
-      <c r="D5">
-        <v>0.28</v>
-      </c>
-      <c r="E5">
-        <v>0.256</v>
-      </c>
-      <c r="F5">
-        <v>0.485</v>
-      </c>
-      <c r="G5">
-        <v>1.365</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6">
-        <v>0.828</v>
-      </c>
-      <c r="C6">
-        <v>1.69</v>
-      </c>
-      <c r="D6">
-        <v>1.091</v>
-      </c>
-      <c r="E6">
-        <v>1.091</v>
-      </c>
-      <c r="F6">
-        <v>0.137</v>
-      </c>
-      <c r="G6">
-        <v>0.05</v>
       </c>
     </row>
   </sheetData>
@@ -1489,104 +1477,65 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="5" outlineLevelCol="5"/>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="2" outlineLevelCol="5"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="B1">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1">
         <v>800</v>
       </c>
-      <c r="C1">
+      <c r="C1" s="1">
         <v>900</v>
       </c>
-      <c r="D1">
+      <c r="D1" s="1">
         <v>1000</v>
       </c>
-      <c r="E1">
+      <c r="E1" s="1">
         <v>1100</v>
       </c>
-      <c r="F1">
+      <c r="F1" s="1">
         <v>1200</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="2">
         <v>0.284</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="2">
         <v>0.299</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="3">
         <v>0.485</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>0.475</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2" s="2">
         <v>0.434</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="1">
+      <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="2">
         <v>1.336</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="2">
         <v>1.586</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="3">
         <v>1.689</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>1.481</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3" s="2">
         <v>1.398</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5">
-        <v>0.485</v>
-      </c>
-      <c r="C5">
-        <v>0.485</v>
-      </c>
-      <c r="D5">
-        <v>0.485</v>
-      </c>
-      <c r="E5">
-        <v>0.485</v>
-      </c>
-      <c r="F5">
-        <v>0.437</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6">
-        <v>1.63</v>
-      </c>
-      <c r="C6">
-        <v>1.587</v>
-      </c>
-      <c r="D6">
-        <v>1.69</v>
-      </c>
-      <c r="E6">
-        <v>1.481</v>
-      </c>
-      <c r="F6">
-        <v>1.499</v>
       </c>
     </row>
   </sheetData>
@@ -1598,104 +1547,65 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="5" outlineLevelCol="5"/>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="2" outlineLevelCol="5"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="B1">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1">
         <v>4</v>
       </c>
-      <c r="C1">
+      <c r="C1" s="1">
         <v>5</v>
       </c>
-      <c r="D1">
+      <c r="D1" s="1">
         <v>6</v>
       </c>
-      <c r="E1">
+      <c r="E1" s="1">
         <v>7</v>
       </c>
-      <c r="F1">
+      <c r="F1" s="1">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="1">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="2">
         <v>0.414</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="2">
         <v>0.431</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="3">
         <v>0.485</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>0.315</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2" s="2">
         <v>0.269</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="1">
+      <c r="A3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="2">
         <v>0.675</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="3">
         <v>1.689</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="2">
         <v>1.387</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>1.456</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3" s="2">
         <v>0.978</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5">
-        <v>0.485</v>
-      </c>
-      <c r="C5">
-        <v>0.485</v>
-      </c>
-      <c r="D5">
-        <v>0.485</v>
-      </c>
-      <c r="E5">
-        <v>0.485</v>
-      </c>
-      <c r="F5">
-        <v>0.485</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6">
-        <v>0.676</v>
-      </c>
-      <c r="C6">
-        <v>1.69</v>
-      </c>
-      <c r="D6">
-        <v>1.388</v>
-      </c>
-      <c r="E6">
-        <v>1.388</v>
-      </c>
-      <c r="F6">
-        <v>0.979</v>
       </c>
     </row>
   </sheetData>

</xml_diff>